<commit_message>
árlista rg pc, és szerver még hiányzik.
a laptop és a pc kapott külön munkalapot.
</commit_message>
<xml_diff>
--- a/CoreLink-KFT árlista.xlsx
+++ b/CoreLink-KFT árlista.xlsx
@@ -1,42 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TÜRR\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D39A20-8AA8-41C3-BC7F-B1DA4F74634C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D37CEABD-C506-4DF9-AE75-3F399686666D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{0916B2E3-0F4C-4406-9F9F-122E188C2873}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11385" xr2:uid="{0916B2E3-0F4C-4406-9F9F-122E188C2873}"/>
   </bookViews>
   <sheets>
-    <sheet name="Munka1" sheetId="1" r:id="rId1"/>
+    <sheet name="Össz." sheetId="1" r:id="rId1"/>
+    <sheet name="Pc" sheetId="3" r:id="rId2"/>
+    <sheet name="Laptop" sheetId="2" r:id="rId3"/>
+    <sheet name="Szerver" sheetId="5" r:id="rId4"/>
+    <sheet name="ASA" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
   <si>
     <t>Eszköz</t>
   </si>
@@ -117,13 +110,77 @@
   </si>
   <si>
     <t>1000m</t>
+  </si>
+  <si>
+    <t>Processzor</t>
+  </si>
+  <si>
+    <t>amd ryzen 5 5500gt</t>
+  </si>
+  <si>
+    <t>Alaplap</t>
+  </si>
+  <si>
+    <t>asrock b450m pro4 r2.0</t>
+  </si>
+  <si>
+    <t>Ár</t>
+  </si>
+  <si>
+    <t>RAM</t>
+  </si>
+  <si>
+    <t>8GB DDR4</t>
+  </si>
+  <si>
+    <t>SSD</t>
+  </si>
+  <si>
+    <t>western digital wd red sa500 nas 500gb</t>
+  </si>
+  <si>
+    <t>Tápegység</t>
+  </si>
+  <si>
+    <t>Gépház</t>
+  </si>
+  <si>
+    <t>whiteshark panzer-2</t>
+  </si>
+  <si>
+    <t>deepcool 650w - pf650</t>
+  </si>
+  <si>
+    <t>Összesen:</t>
+  </si>
+  <si>
+    <t>lenovo ideapad slim 5 14arp10</t>
+  </si>
+  <si>
+    <t>Modell</t>
+  </si>
+  <si>
+    <t>Belső részek</t>
+  </si>
+  <si>
+    <t>Belső részek modellje</t>
+  </si>
+  <si>
+    <t>https://psref.lenovo.com/Product/IdeaPad/IdeaPad_Slim_5_14ARP10</t>
+  </si>
+  <si>
+    <t>Specifikációk (link):</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
+    <numFmt numFmtId="165" formatCode="#,##0\ [$€-1];[Red]\-#,##0\ [$€-1]"/>
+  </numFmts>
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -153,8 +210,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
@@ -489,19 +551,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC3A488-0522-4B95-8ABB-90B3293D8594}">
-  <dimension ref="A2:G17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:G16"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="24.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.25" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -524,7 +586,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -541,15 +603,15 @@
         <v>4</v>
       </c>
       <c r="F3">
-        <f>B3+C3+D3+E3</f>
+        <f t="shared" ref="F3:F14" si="0">B3+C3+D3+E3</f>
         <v>21</v>
       </c>
       <c r="G3">
-        <f>F3*475</f>
-        <v>9975</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F3*465.34</f>
+        <v>9772.14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4" t="s">
         <v>15</v>
       </c>
@@ -566,15 +628,11 @@
         <v>1</v>
       </c>
       <c r="F4">
-        <f>B4+C4+D4+E4</f>
-        <v>4</v>
-      </c>
-      <c r="G4">
-        <f>F4*710</f>
-        <v>2840</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -591,15 +649,15 @@
         <v>0</v>
       </c>
       <c r="F5">
-        <f>B5+C5+D5+E5</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="G5">
-        <f>F5*565</f>
-        <v>3390</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+        <f>6*645.34</f>
+        <v>3872.04</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -616,15 +674,15 @@
         <v>4</v>
       </c>
       <c r="F6">
-        <f>B6+C6+D6+E6</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="G6">
-        <f>F6*25</f>
-        <v>500</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F6*30</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -641,15 +699,15 @@
         <v>4</v>
       </c>
       <c r="F7">
-        <f>B7+C7+D7+E7</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="G7">
-        <f>F7*50</f>
-        <v>850</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F7*55</f>
+        <v>935</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -666,15 +724,15 @@
         <v>5</v>
       </c>
       <c r="F8">
-        <f>B8+C8+D8+E8</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="G8">
-        <f>F8*55</f>
-        <v>1265</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F8*60</f>
+        <v>1380</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -691,15 +749,15 @@
         <v>2</v>
       </c>
       <c r="F9">
-        <f>B9+C9+D9+E9</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="G9">
-        <f>F9*390</f>
-        <v>5070</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F9*400</f>
+        <v>5200</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -716,15 +774,15 @@
         <v>1</v>
       </c>
       <c r="F10">
-        <f>B10+C10+D10+E10</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="G10">
-        <f>F10*240</f>
-        <v>480</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F10*250</f>
+        <v>500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -741,15 +799,11 @@
         <v>1</v>
       </c>
       <c r="F11">
-        <f>B11+C11+D11+E11</f>
-        <v>4</v>
-      </c>
-      <c r="G11">
-        <f>F11*2600</f>
-        <v>10400</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -766,15 +820,15 @@
         <v>0</v>
       </c>
       <c r="F12">
-        <f>B12+C12+D12+E12</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G12">
-        <f>F12*265</f>
-        <v>265</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F12*300</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -791,15 +845,15 @@
         <v>0</v>
       </c>
       <c r="F13">
-        <f>B13+C13+D13+E13</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="G13">
-        <f>F13*840</f>
-        <v>840</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F13*1000</f>
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -816,15 +870,15 @@
         <v>0</v>
       </c>
       <c r="F14">
-        <f>B14+C14+D14+E14</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="G14">
-        <f>F14*80</f>
-        <v>240</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+        <f>F14*95</f>
+        <v>285</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -847,7 +901,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7">
       <c r="A16" t="s">
         <v>6</v>
       </c>
@@ -868,15 +922,165 @@
       </c>
       <c r="G16">
         <v>750</v>
-      </c>
-    </row>
-    <row r="17" spans="7:7" x14ac:dyDescent="0.3">
-      <c r="G17">
-        <f>G3+G4+G5+G6+G7+G8+G9+G10+G11+G12+G13+G14+G15+G16</f>
-        <v>37165</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA031806-A867-4AB7-87A5-188388593F64}">
+  <dimension ref="B2:D9"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.75" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:4">
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4">
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="1">
+        <v>133.34</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4">
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D4" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4">
+      <c r="B5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4">
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4">
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="2">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4">
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4">
+      <c r="C9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="1">
+        <f>D3+D4+D5+D6+D7+D8</f>
+        <v>465.34000000000003</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{093B1946-6DF5-47CD-A15C-97F472879888}">
+  <dimension ref="A2:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col min="1" max="1" width="16.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3">
+      <c r="C2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="1">
+        <v>645.34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CA35558-1128-46F2-B5D0-284A6299A096}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B02CC2-4B7C-42D0-8DA7-565399B726A1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Árlista a specifikációkkal és munkalapokkal.
</commit_message>
<xml_diff>
--- a/CoreLink-KFT árlista.xlsx
+++ b/CoreLink-KFT árlista.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TÜRR\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D37CEABD-C506-4DF9-AE75-3F399686666D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4DA5B8-E9F2-4D3B-8C85-0F87AD6E09B8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11385" xr2:uid="{0916B2E3-0F4C-4406-9F9F-122E188C2873}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Pc" sheetId="3" r:id="rId2"/>
     <sheet name="Laptop" sheetId="2" r:id="rId3"/>
     <sheet name="Szerver" sheetId="5" r:id="rId4"/>
-    <sheet name="ASA" sheetId="6" r:id="rId5"/>
+    <sheet name="ASA" sheetId="6" state="hidden" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="58">
   <si>
     <t>Eszköz</t>
   </si>
@@ -94,9 +94,6 @@
     <t>AP</t>
   </si>
   <si>
-    <t>Szerver</t>
-  </si>
-  <si>
     <t>90m</t>
   </si>
   <si>
@@ -170,6 +167,42 @@
   </si>
   <si>
     <t>Specifikációk (link):</t>
+  </si>
+  <si>
+    <t>IRODAI!!</t>
+  </si>
+  <si>
+    <t>Rendszegazda</t>
+  </si>
+  <si>
+    <t>Ryzen 7 9700X</t>
+  </si>
+  <si>
+    <t>32GB DDR5</t>
+  </si>
+  <si>
+    <t>1TB</t>
+  </si>
+  <si>
+    <t>Corsair RM650e</t>
+  </si>
+  <si>
+    <t>Lian Li O11D Mini V2</t>
+  </si>
+  <si>
+    <t>MSI MAG B850</t>
+  </si>
+  <si>
+    <t>DELL PowerEdge T560 Tower H755 (HW RAID 0,1,5,10,50,60) 1x 4510 2x PSU iDRAC</t>
+  </si>
+  <si>
+    <t>Szerver fizikai (összesen 2)</t>
+  </si>
+  <si>
+    <t>Windows és linux szerverszolgáltatás(összesen 2)</t>
+  </si>
+  <si>
+    <t>összesen:</t>
   </si>
 </sst>
 </file>
@@ -180,10 +213,34 @@
     <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
     <numFmt numFmtId="165" formatCode="#,##0\ [$€-1];[Red]\-#,##0\ [$€-1]"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF343B43"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="238"/>
@@ -207,18 +264,29 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hivatkozás" xfId="1" builtinId="8"/>
     <cellStyle name="Normál" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -232,6 +300,72 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>674650</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>122463</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>585107</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>115660</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Kép 1" descr="IdeaPad_Slim_5_14ARP10_CT1_01.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{61C72975-010B-4518-A987-72C016D34D45}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="7056400" y="299356"/>
+          <a:ext cx="4672957" cy="3707947"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -551,10 +685,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC3A488-0522-4B95-8ABB-90B3293D8594}">
-  <dimension ref="A2:G16"/>
+  <dimension ref="A2:G18"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="24.75" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="43.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.5" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
@@ -603,10 +737,10 @@
         <v>4</v>
       </c>
       <c r="F3">
-        <f t="shared" ref="F3:F14" si="0">B3+C3+D3+E3</f>
+        <f t="shared" ref="F3:F15" si="0">B3+C3+D3+E3</f>
         <v>21</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="8">
         <f>F3*465.34</f>
         <v>9772.14</v>
       </c>
@@ -631,6 +765,10 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
+      <c r="G4" s="8">
+        <f>1383.29*F4</f>
+        <v>5533.16</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -652,7 +790,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="8">
         <f>6*645.34</f>
         <v>3872.04</v>
       </c>
@@ -677,7 +815,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="8">
         <f>F6*30</f>
         <v>600</v>
       </c>
@@ -702,7 +840,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="8">
         <f>F7*55</f>
         <v>935</v>
       </c>
@@ -727,7 +865,7 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="8">
         <f>F8*60</f>
         <v>1380</v>
       </c>
@@ -752,7 +890,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="G9">
+      <c r="G9" s="8">
         <f>F9*400</f>
         <v>5200</v>
       </c>
@@ -777,60 +915,62 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="8">
         <f>F10*250</f>
         <v>500</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11">
-        <f t="shared" si="0"/>
-        <v>4</v>
+        <v>2</v>
+      </c>
+      <c r="G11" s="8">
+        <f>27162.5*2</f>
+        <v>54325</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12">
         <v>0</v>
       </c>
       <c r="F12">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="G12">
-        <f>F12*300</f>
-        <v>300</v>
+        <v>2</v>
+      </c>
+      <c r="G12" s="8">
+        <f>F12*1383.29</f>
+        <v>2766.58</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -848,17 +988,17 @@
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G13">
-        <f>F13*1000</f>
-        <v>1000</v>
+      <c r="G13" s="8">
+        <f>F13*300</f>
+        <v>300</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -871,57 +1011,91 @@
       </c>
       <c r="F14">
         <f t="shared" si="0"/>
-        <v>3</v>
-      </c>
-      <c r="G14">
-        <f>F14*95</f>
-        <v>285</v>
+        <v>1</v>
+      </c>
+      <c r="G14" s="8">
+        <f>F14*1000</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="A15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C15" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" t="s">
-        <v>23</v>
-      </c>
-      <c r="E15" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" t="s">
-        <v>24</v>
-      </c>
-      <c r="G15">
-        <v>300</v>
+        <v>20</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="G15" s="8">
+        <f>F15*95</f>
+        <v>285</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" t="s">
+        <v>22</v>
+      </c>
+      <c r="E16" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" s="8">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
         <v>6</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" t="s">
         <v>25</v>
       </c>
-      <c r="C16" t="s">
-        <v>17</v>
-      </c>
-      <c r="D16" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" t="s">
-        <v>17</v>
-      </c>
-      <c r="F16" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16">
+      <c r="G17" s="8">
         <v>750</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="F18" t="s">
+        <v>57</v>
+      </c>
+      <c r="G18" s="8">
+        <f>G17+G16+G15+G14+G13+G12+G11+G10+G9+G8+G7+G6+G5+G4+G3</f>
+        <v>87518.92</v>
       </c>
     </row>
   </sheetData>
@@ -931,101 +1105,200 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA031806-A867-4AB7-87A5-188388593F64}">
-  <dimension ref="B2:D9"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
+    <col min="1" max="1" width="13.375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33.75" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4">
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s">
         <v>43</v>
       </c>
-      <c r="C2" t="s">
-        <v>44</v>
-      </c>
       <c r="D2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="2:4">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
         <v>27</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
       </c>
       <c r="D3" s="1">
         <v>133.34</v>
       </c>
     </row>
-    <row r="4" spans="2:4">
+    <row r="4" spans="1:4">
       <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
         <v>29</v>
-      </c>
-      <c r="C4" t="s">
-        <v>30</v>
       </c>
       <c r="D4" s="2">
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="2:4">
+    <row r="5" spans="1:4">
       <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
         <v>32</v>
-      </c>
-      <c r="C5" t="s">
-        <v>33</v>
       </c>
       <c r="D5" s="2">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="2:4">
+    <row r="6" spans="1:4">
       <c r="B6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" t="s">
         <v>34</v>
-      </c>
-      <c r="C6" t="s">
-        <v>35</v>
       </c>
       <c r="D6" s="2">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="2:4">
+    <row r="7" spans="1:4">
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" s="2">
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="2:4">
+    <row r="8" spans="1:4">
       <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
         <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>38</v>
       </c>
       <c r="D8" s="2">
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="2:4">
+    <row r="9" spans="1:4">
       <c r="C9" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D9" s="1">
         <f>D3+D4+D5+D6+D7+D8</f>
         <v>465.34000000000003</v>
       </c>
     </row>
+    <row r="12" spans="1:4">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="B13" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15">
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="1">
+        <v>319.91000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="B15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="1">
+        <v>226.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" t="s">
+        <v>49</v>
+      </c>
+      <c r="D16" s="1">
+        <v>533.17999999999995</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4">
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="1">
+        <v>140.19999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4">
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="2">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="14.25" customHeight="1">
+      <c r="B19" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="1">
+        <v>83.4</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4">
+      <c r="C20" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D20" s="1">
+        <f>D14+D15+D16+D17+D18+D19</f>
+        <v>1383.2900000000002</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1040,15 +1313,15 @@
   <sheetData>
     <row r="2" spans="1:3">
       <c r="C2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" s="1">
         <v>645.34</v>
@@ -1056,22 +1329,48 @@
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" t="s">
         <v>45</v>
       </c>
+      <c r="B4" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{088442AC-7931-4CD2-B346-F48B48466A88}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CA35558-1128-46F2-B5D0-284A6299A096}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="124" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="20.100000000000001" customHeight="1">
+      <c r="A1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="46.5">
+      <c r="A2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="1">
+        <v>27162.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="14.25" customHeight="1"/>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
debrecen topologia, ip cimek portokkal, arlista
</commit_message>
<xml_diff>
--- a/CoreLink-KFT árlista.xlsx
+++ b/CoreLink-KFT árlista.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TÜRR\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4DA5B8-E9F2-4D3B-8C85-0F87AD6E09B8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F538E35-FE9F-4BD4-B6EA-103AB0DD792C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11385" xr2:uid="{0916B2E3-0F4C-4406-9F9F-122E188C2873}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{0916B2E3-0F4C-4406-9F9F-122E188C2873}"/>
   </bookViews>
   <sheets>
     <sheet name="Össz." sheetId="1" r:id="rId1"/>
@@ -24,12 +24,23 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="62">
   <si>
     <t>Eszköz</t>
   </si>
@@ -193,9 +204,6 @@
     <t>MSI MAG B850</t>
   </si>
   <si>
-    <t>DELL PowerEdge T560 Tower H755 (HW RAID 0,1,5,10,50,60) 1x 4510 2x PSU iDRAC</t>
-  </si>
-  <si>
     <t>Szerver fizikai (összesen 2)</t>
   </si>
   <si>
@@ -203,6 +211,21 @@
   </si>
   <si>
     <t>összesen:</t>
+  </si>
+  <si>
+    <t>AMD Ryzen™ 7 7735HS</t>
+  </si>
+  <si>
+    <t>Integralt videokártya</t>
+  </si>
+  <si>
+    <t>AMD Radeon™ 680M</t>
+  </si>
+  <si>
+    <t>DELL PowerEdge R760XS 2U Rack H755 (HW RAID 0,1,5,10,50,60) 1x 4514Y 2x PSU iDRAC9 Enterprise 12x 3,5</t>
+  </si>
+  <si>
+    <t>https://tinyurl.com/286yypwa</t>
   </si>
 </sst>
 </file>
@@ -211,9 +234,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.00\ [$€-1];[Red]\-#,##0.00\ [$€-1]"/>
-    <numFmt numFmtId="165" formatCode="#,##0\ [$€-1];[Red]\-#,##0\ [$€-1]"/>
+    <numFmt numFmtId="165" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-;_-@_-"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -221,13 +244,6 @@
       <family val="2"/>
       <charset val="238"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF0A0A0A"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="238"/>
     </font>
     <font>
       <b/>
@@ -246,16 +262,71 @@
       <charset val="238"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF646363"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF646363"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -263,27 +334,58 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hivatkozás" xfId="1" builtinId="8"/>
@@ -306,16 +408,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>674650</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>422877</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>122463</xdr:rowOff>
+      <xdr:rowOff>130630</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>585107</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>115660</xdr:rowOff>
+      <xdr:colOff>478971</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>7405</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -345,8 +447,74 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="7056400" y="299356"/>
-          <a:ext cx="4672957" cy="3707947"/>
+          <a:off x="7172020" y="315687"/>
+          <a:ext cx="3713694" cy="3392861"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>160020</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>186620</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>182879</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Kép 2" descr="DELL PowerEdge R760XS 2U Rack H755 (HW RAID 0,1,5,10,50,60) 1x 4514Y 2x PSU iDRAC9 Enterprise 12x 3,5 EMEA_PER760XS4SPL_CN37055_256GBS4X4000SSD_S large">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D40CE83F-2509-C800-7769-DEAF69B7D979}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="5745480" y="186620"/>
+          <a:ext cx="5509259" cy="1596460"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -686,416 +854,421 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FBC3A488-0522-4B95-8ABB-90B3293D8594}">
   <dimension ref="A2:G18"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="43.25" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.25" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="43.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.21875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.875" customWidth="1"/>
+    <col min="7" max="7" width="13.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="2">
         <v>7</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="2">
         <v>6</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <v>4</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>4</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <f t="shared" ref="F3:F15" si="0">B3+C3+D3+E3</f>
         <v>21</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="13">
         <f>F3*465.34</f>
         <v>9772.14</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="2">
         <v>1</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="2">
         <v>1</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>1</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <v>1</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="G4" s="8">
+      <c r="G4" s="13">
         <f>1383.29*F4</f>
         <v>5533.16</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="2">
         <v>1</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="2">
         <v>5</v>
       </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
+      <c r="D5" s="2">
+        <v>0</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0</v>
+      </c>
+      <c r="F5" s="2">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="G5" s="8">
+      <c r="G5" s="13">
         <f>6*645.34</f>
         <v>3872.04</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="2">
         <v>8</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="2">
         <v>4</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>4</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>4</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="G6" s="8">
+      <c r="G6" s="13">
         <f>F6*30</f>
         <v>600</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="2">
         <v>7</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="2">
         <v>2</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>4</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="2">
         <v>4</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="G7" s="8">
+      <c r="G7" s="13">
         <f>F7*55</f>
         <v>935</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B8">
+      <c r="B8" s="2">
         <v>8</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="2">
         <v>4</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>6</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="2">
         <v>5</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="2">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="G8" s="8">
+      <c r="G8" s="13">
         <f>F8*60</f>
         <v>1380</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="2">
         <v>4</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="2">
         <v>4</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="2">
         <v>3</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="2">
         <v>2</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="2">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="G9" s="8">
+      <c r="G9" s="13">
         <f>F9*400</f>
         <v>5200</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-      <c r="C10">
+      <c r="B10" s="2">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2">
         <v>1</v>
       </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2">
         <v>1</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="2">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="G10" s="8">
+      <c r="G10" s="13">
         <f>F10*250</f>
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2">
+        <v>2</v>
+      </c>
+      <c r="G11" s="13">
+        <f>26561.24*2</f>
+        <v>53122.48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B11">
+      <c r="B12" s="2">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2">
         <v>1</v>
       </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
+      <c r="D12" s="2">
         <v>1</v>
       </c>
-      <c r="F11">
+      <c r="E12" s="2">
+        <v>0</v>
+      </c>
+      <c r="F12" s="2">
         <v>2</v>
       </c>
-      <c r="G11" s="8">
-        <f>27162.5*2</f>
-        <v>54325</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>56</v>
-      </c>
-      <c r="B12">
-        <v>0</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>2</v>
-      </c>
-      <c r="G12" s="8">
+      <c r="G12" s="13">
         <f>F12*1383.29</f>
         <v>2766.58</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="2">
         <v>1</v>
       </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>0</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
+      <c r="C13" s="2">
+        <v>0</v>
+      </c>
+      <c r="D13" s="2">
+        <v>0</v>
+      </c>
+      <c r="E13" s="2">
+        <v>0</v>
+      </c>
+      <c r="F13" s="2">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G13" s="8">
+      <c r="G13" s="13">
         <f>F13*300</f>
         <v>300</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="2">
         <v>1</v>
       </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14">
+      <c r="C14" s="2">
+        <v>0</v>
+      </c>
+      <c r="D14" s="2">
+        <v>0</v>
+      </c>
+      <c r="E14" s="2">
+        <v>0</v>
+      </c>
+      <c r="F14" s="2">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="G14" s="8">
+      <c r="G14" s="13">
         <f>F14*1000</f>
         <v>1000</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="2">
         <v>3</v>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
+      <c r="C15" s="2">
+        <v>0</v>
+      </c>
+      <c r="D15" s="2">
+        <v>0</v>
+      </c>
+      <c r="E15" s="2">
+        <v>0</v>
+      </c>
+      <c r="F15" s="2">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="G15" s="8">
+      <c r="G15" s="13">
         <f>F15*95</f>
         <v>285</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G16" s="8">
+      <c r="G16" s="13">
         <v>300</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="G17" s="8">
+      <c r="G17" s="13">
         <v>750</v>
       </c>
     </row>
-    <row r="18" spans="1:7">
-      <c r="F18" t="s">
-        <v>57</v>
-      </c>
-      <c r="G18" s="8">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G18" s="15">
         <f>G17+G16+G15+G14+G13+G12+G11+G10+G9+G8+G7+G6+G5+G4+G3</f>
-        <v>87518.92</v>
+        <v>86316.4</v>
       </c>
     </row>
   </sheetData>
@@ -1106,192 +1279,227 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA031806-A867-4AB7-87A5-188388593F64}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="B3" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="3"/>
+      <c r="B3" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="17">
         <v>133.34</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="B4" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3"/>
+      <c r="B4" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="17">
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="B5" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+      <c r="B5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="17">
         <v>68</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="B6" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="3"/>
+      <c r="B6" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="17">
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="B7" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="3"/>
+      <c r="B7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="17">
         <v>55</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="B8" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3"/>
+      <c r="B8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="17">
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="C9" s="3" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="15">
         <f>D3+D4+D5+D6+D7+D8</f>
         <v>465.34000000000003</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="B13" t="s">
+      <c r="B13" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="15">
-      <c r="B14" t="s">
+    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="3"/>
+      <c r="B14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="17">
         <v>319.91000000000003</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="B15" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="3"/>
+      <c r="B15" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="17">
         <v>226.6</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
-      <c r="B16" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="3"/>
+      <c r="B16" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="17">
         <v>533.17999999999995</v>
       </c>
     </row>
-    <row r="17" spans="2:4">
-      <c r="B17" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="3"/>
+      <c r="B17" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="17">
         <v>140.19999999999999</v>
       </c>
     </row>
-    <row r="18" spans="2:4">
-      <c r="B18" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="3"/>
+      <c r="B18" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="17">
         <v>80</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="14.25" customHeight="1">
-      <c r="B19" t="s">
+    <row r="19" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="3"/>
+      <c r="B19" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="17">
         <v>83.4</v>
       </c>
     </row>
-    <row r="20" spans="2:4">
-      <c r="C20" s="3" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="3"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="15">
         <f>D14+D15+D16+D17+D18+D19</f>
         <v>1383.2900000000002</v>
       </c>
@@ -1304,36 +1512,74 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{093B1946-6DF5-47CD-A15C-97F472879888}">
-  <dimension ref="A2:C4"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A2:C9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="22.21875" customWidth="1"/>
+    <col min="2" max="2" width="58.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="C2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="4">
         <v>645.34</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="9" t="s">
         <v>44</v>
       </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="3"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1347,38 +1593,47 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CA35558-1128-46F2-B5D0-284A6299A096}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="124" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61" customWidth="1"/>
+    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="20.100000000000001" customHeight="1">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:2" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="46.5">
-      <c r="A2" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="1">
-        <v>27162.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="14.25" customHeight="1"/>
+    <row r="2" spans="1:2" ht="94.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="16">
+        <v>26561.24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="1"/>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" xr:uid="{E27FA90F-7B6A-4E69-9FBC-1B7D8BEEC723}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97B02CC2-4B7C-42D0-8DA7-565399B726A1}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>